<commit_message>
feat: add charts to Catamarca dashboard workbook
</commit_message>
<xml_diff>
--- a/catamarca_creditos/analisis_cartera_catamarca.xlsx
+++ b/catamarca_creditos/analisis_cartera_catamarca.xlsx
@@ -207,6 +207,223 @@
     </indexedColors>
   </colors>
 </styleSheet>
+</file>
+
+<file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <style val="10"/>
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>Estado de cartera al corte marzo 2026</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <barChart>
+        <barDir val="col"/>
+        <grouping val="clustered"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <strRef>
+              <f>'Dashboard'!B20</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'Dashboard'!$A$21:$A$24</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Dashboard'!$B$21:$B$24</f>
+            </numRef>
+          </val>
+        </ser>
+        <gapWidth val="150"/>
+        <axId val="10"/>
+        <axId val="100"/>
+      </barChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Estado</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Cantidad de créditos</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <style val="10"/>
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>Semáforo de cartera</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <pieChart>
+        <varyColors val="1"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <strRef>
+              <f>'Dashboard'!E20</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'Dashboard'!$D$21:$D$23</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Dashboard'!$E$21:$E$23</f>
+            </numRef>
+          </val>
+        </ser>
+        <firstSliceAng val="0"/>
+      </pieChart>
+    </plotArea>
+    <legend>
+      <legendPos val="r"/>
+    </legend>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
+      <col>6</col>
+      <colOff>0</colOff>
+      <row>1</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="5760000" cy="2880000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="1" name="Chart 1"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>6</col>
+      <colOff>0</colOff>
+      <row>19</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="4320000" cy="2880000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="2" name="Chart 2"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -553,7 +770,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E13"/>
+  <dimension ref="A1:E25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -739,11 +956,106 @@
         <v>0.3641975308641975</v>
       </c>
     </row>
+    <row r="14"/>
+    <row r="20" hidden="1">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Categoría</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Cantidad</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>Semáforo</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>Cantidad</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" hidden="1">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Con cobro en marzo</t>
+        </is>
+      </c>
+      <c r="B21" t="n">
+        <v>8740000</v>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>Verde</t>
+        </is>
+      </c>
+      <c r="E21" t="n">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="22" hidden="1">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Cancelados / finalizados</t>
+        </is>
+      </c>
+      <c r="B22" t="n">
+        <v>23</v>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>Amarillo</t>
+        </is>
+      </c>
+      <c r="E22" t="n">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="23" hidden="1">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Sin cobro en marzo</t>
+        </is>
+      </c>
+      <c r="B23" t="n">
+        <v>59</v>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>Rojo</t>
+        </is>
+      </c>
+      <c r="E23" t="n">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="24" hidden="1">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Sin registro en marzo</t>
+        </is>
+      </c>
+      <c r="B24" t="n">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Mora operativa</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:D1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
fix: rebuild dashboard charts with visible data ranges
</commit_message>
<xml_diff>
--- a/catamarca_creditos/analisis_cartera_catamarca.xlsx
+++ b/catamarca_creditos/analisis_cartera_catamarca.xlsx
@@ -23,7 +23,7 @@
     <numFmt numFmtId="164" formatCode="$ #,##0.00"/>
     <numFmt numFmtId="165" formatCode="yyyy-mm-dd"/>
   </numFmts>
-  <fonts count="4">
+  <fonts count="5">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -42,6 +42,9 @@
     <font>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
+    </font>
+    <font>
+      <color rgb="00000000"/>
     </font>
   </fonts>
   <fills count="7">
@@ -103,7 +106,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -123,6 +126,8 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -230,14 +235,14 @@
     </title>
     <plotArea>
       <barChart>
-        <barDir val="col"/>
+        <barDir val="bar"/>
         <grouping val="clustered"/>
         <ser>
           <idx val="0"/>
           <order val="0"/>
           <tx>
             <strRef>
-              <f>'Dashboard'!B20</f>
+              <f>'Dashboard'!I3</f>
             </strRef>
           </tx>
           <spPr>
@@ -247,12 +252,12 @@
           </spPr>
           <cat>
             <numRef>
-              <f>'Dashboard'!$A$21:$A$24</f>
+              <f>'Dashboard'!$H$4:$H$7</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Dashboard'!$B$21:$B$24</f>
+              <f>'Dashboard'!$I$4:$I$7</f>
             </numRef>
           </val>
         </ser>
@@ -275,7 +280,7 @@
                   <a:defRPr/>
                 </a:pPr>
                 <a:r>
-                  <a:t>Estado</a:t>
+                  <a:t>Cantidad</a:t>
                 </a:r>
               </a:p>
             </rich>
@@ -302,7 +307,7 @@
                   <a:defRPr/>
                 </a:pPr>
                 <a:r>
-                  <a:t>Cantidad de créditos</a:t>
+                  <a:t>Estado</a:t>
                 </a:r>
               </a:p>
             </rich>
@@ -346,7 +351,7 @@
           <order val="0"/>
           <tx>
             <strRef>
-              <f>'Dashboard'!E20</f>
+              <f>'Dashboard'!I11</f>
             </strRef>
           </tx>
           <spPr>
@@ -356,12 +361,12 @@
           </spPr>
           <cat>
             <numRef>
-              <f>'Dashboard'!$D$21:$D$23</f>
+              <f>'Dashboard'!$H$12:$H$14</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Dashboard'!$E$21:$E$23</f>
+              <f>'Dashboard'!$I$12:$I$14</f>
             </numRef>
           </val>
         </ser>
@@ -381,12 +386,12 @@
 <wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
-      <col>6</col>
+      <col>10</col>
       <colOff>0</colOff>
       <row>1</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="5760000" cy="2880000"/>
+    <ext cx="4320000" cy="2520000"/>
     <graphicFrame>
       <nvGraphicFramePr>
         <cNvPr id="1" name="Chart 1"/>
@@ -403,12 +408,12 @@
   </oneCellAnchor>
   <oneCellAnchor>
     <from>
-      <col>6</col>
+      <col>10</col>
       <colOff>0</colOff>
-      <row>19</row>
+      <row>17</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="4320000" cy="2880000"/>
+    <ext cx="3600000" cy="2520000"/>
     <graphicFrame>
       <nvGraphicFramePr>
         <cNvPr id="2" name="Chart 2"/>
@@ -770,7 +775,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E25"/>
+  <dimension ref="A1:M25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -778,6 +783,8 @@
     <col width="4" customWidth="1" min="3" max="3"/>
     <col width="28" customWidth="1" min="4" max="4"/>
     <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="24" customWidth="1" min="8" max="8"/>
+    <col width="12" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -798,6 +805,16 @@
           <t>Cruce entre Excel de depósitos y Excel de cobranzas Cecilia</t>
         </is>
       </c>
+      <c r="H2" s="15" t="inlineStr">
+        <is>
+          <t>Base gráfico estados</t>
+        </is>
+      </c>
+      <c r="I2" s="16" t="n"/>
+      <c r="J2" s="16" t="n"/>
+      <c r="K2" s="16" t="n"/>
+      <c r="L2" s="16" t="n"/>
+      <c r="M2" s="16" t="n"/>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -810,6 +827,20 @@
           <t>Créditos desde 2025-12-01 y lectura de cobranza hasta marzo 2026</t>
         </is>
       </c>
+      <c r="H3" s="5" t="inlineStr">
+        <is>
+          <t>Estado</t>
+        </is>
+      </c>
+      <c r="I3" s="5" t="inlineStr">
+        <is>
+          <t>Cantidad</t>
+        </is>
+      </c>
+      <c r="J3" s="16" t="n"/>
+      <c r="K3" s="16" t="n"/>
+      <c r="L3" s="16" t="n"/>
+      <c r="M3" s="16" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -822,6 +853,32 @@
           <t>VERDE = al día / con cobro o finalizado | AMARILLO = sin exigibilidad clara | ROJO = mora operativa</t>
         </is>
       </c>
+      <c r="H4" s="16" t="inlineStr">
+        <is>
+          <t>Con cobro en marzo</t>
+        </is>
+      </c>
+      <c r="I4" s="16" t="n">
+        <v>59</v>
+      </c>
+      <c r="J4" s="16" t="n"/>
+      <c r="K4" s="16" t="n"/>
+      <c r="L4" s="16" t="n"/>
+      <c r="M4" s="16" t="n"/>
+    </row>
+    <row r="5">
+      <c r="H5" s="16" t="inlineStr">
+        <is>
+          <t>Cancelados / finalizados</t>
+        </is>
+      </c>
+      <c r="I5" s="16" t="n">
+        <v>23</v>
+      </c>
+      <c r="J5" s="16" t="n"/>
+      <c r="K5" s="16" t="n"/>
+      <c r="L5" s="16" t="n"/>
+      <c r="M5" s="16" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
@@ -837,6 +894,18 @@
           <t>Resumen de estado</t>
         </is>
       </c>
+      <c r="H6" s="16" t="inlineStr">
+        <is>
+          <t>Sin cobro en marzo</t>
+        </is>
+      </c>
+      <c r="I6" s="16" t="n">
+        <v>59</v>
+      </c>
+      <c r="J6" s="16" t="n"/>
+      <c r="K6" s="16" t="n"/>
+      <c r="L6" s="16" t="n"/>
+      <c r="M6" s="16" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
@@ -855,6 +924,18 @@
       <c r="E7" s="4" t="n">
         <v>78</v>
       </c>
+      <c r="H7" s="16" t="inlineStr">
+        <is>
+          <t>Sin registro en marzo</t>
+        </is>
+      </c>
+      <c r="I7" s="16" t="n">
+        <v>25</v>
+      </c>
+      <c r="J7" s="16" t="n"/>
+      <c r="K7" s="16" t="n"/>
+      <c r="L7" s="16" t="n"/>
+      <c r="M7" s="16" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
@@ -873,6 +954,12 @@
       <c r="E8" s="4" t="n">
         <v>25</v>
       </c>
+      <c r="H8" s="16" t="n"/>
+      <c r="I8" s="16" t="n"/>
+      <c r="J8" s="16" t="n"/>
+      <c r="K8" s="16" t="n"/>
+      <c r="L8" s="16" t="n"/>
+      <c r="M8" s="16" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
@@ -891,6 +978,12 @@
       <c r="E9" s="4" t="n">
         <v>59</v>
       </c>
+      <c r="H9" s="16" t="n"/>
+      <c r="I9" s="16" t="n"/>
+      <c r="J9" s="16" t="n"/>
+      <c r="K9" s="16" t="n"/>
+      <c r="L9" s="16" t="n"/>
+      <c r="M9" s="16" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
@@ -909,6 +1002,16 @@
       <c r="E10" s="4" t="n">
         <v>23</v>
       </c>
+      <c r="H10" s="15" t="inlineStr">
+        <is>
+          <t>Base gráfico semáforo</t>
+        </is>
+      </c>
+      <c r="I10" s="16" t="n"/>
+      <c r="J10" s="16" t="n"/>
+      <c r="K10" s="16" t="n"/>
+      <c r="L10" s="16" t="n"/>
+      <c r="M10" s="16" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
@@ -927,6 +1030,20 @@
       <c r="E11" s="4" t="n">
         <v>59</v>
       </c>
+      <c r="H11" s="5" t="inlineStr">
+        <is>
+          <t>Semáforo</t>
+        </is>
+      </c>
+      <c r="I11" s="5" t="inlineStr">
+        <is>
+          <t>Cantidad</t>
+        </is>
+      </c>
+      <c r="J11" s="16" t="n"/>
+      <c r="K11" s="16" t="n"/>
+      <c r="L11" s="16" t="n"/>
+      <c r="M11" s="16" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
@@ -945,6 +1062,18 @@
       <c r="E12" s="4" t="n">
         <v>25</v>
       </c>
+      <c r="H12" s="16" t="inlineStr">
+        <is>
+          <t>Verde</t>
+        </is>
+      </c>
+      <c r="I12" s="16" t="n">
+        <v>78</v>
+      </c>
+      <c r="J12" s="16" t="n"/>
+      <c r="K12" s="16" t="n"/>
+      <c r="L12" s="16" t="n"/>
+      <c r="M12" s="16" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
@@ -955,8 +1084,73 @@
       <c r="B13" s="10" t="n">
         <v>0.3641975308641975</v>
       </c>
-    </row>
-    <row r="14"/>
+      <c r="H13" s="16" t="inlineStr">
+        <is>
+          <t>Amarillo</t>
+        </is>
+      </c>
+      <c r="I13" s="16" t="n">
+        <v>25</v>
+      </c>
+      <c r="J13" s="16" t="n"/>
+      <c r="K13" s="16" t="n"/>
+      <c r="L13" s="16" t="n"/>
+      <c r="M13" s="16" t="n"/>
+    </row>
+    <row r="14">
+      <c r="H14" s="16" t="inlineStr">
+        <is>
+          <t>Rojo</t>
+        </is>
+      </c>
+      <c r="I14" s="16" t="n">
+        <v>59</v>
+      </c>
+      <c r="J14" s="16" t="n"/>
+      <c r="K14" s="16" t="n"/>
+      <c r="L14" s="16" t="n"/>
+      <c r="M14" s="16" t="n"/>
+    </row>
+    <row r="15">
+      <c r="H15" s="16" t="n"/>
+      <c r="I15" s="16" t="n"/>
+      <c r="J15" s="16" t="n"/>
+      <c r="K15" s="16" t="n"/>
+      <c r="L15" s="16" t="n"/>
+      <c r="M15" s="16" t="n"/>
+    </row>
+    <row r="16">
+      <c r="H16" s="16" t="n"/>
+      <c r="I16" s="16" t="n"/>
+      <c r="J16" s="16" t="n"/>
+      <c r="K16" s="16" t="n"/>
+      <c r="L16" s="16" t="n"/>
+      <c r="M16" s="16" t="n"/>
+    </row>
+    <row r="17">
+      <c r="H17" s="16" t="n"/>
+      <c r="I17" s="16" t="n"/>
+      <c r="J17" s="16" t="n"/>
+      <c r="K17" s="16" t="n"/>
+      <c r="L17" s="16" t="n"/>
+      <c r="M17" s="16" t="n"/>
+    </row>
+    <row r="18">
+      <c r="H18" s="16" t="n"/>
+      <c r="I18" s="16" t="n"/>
+      <c r="J18" s="16" t="n"/>
+      <c r="K18" s="16" t="n"/>
+      <c r="L18" s="16" t="n"/>
+      <c r="M18" s="16" t="n"/>
+    </row>
+    <row r="19">
+      <c r="H19" s="16" t="n"/>
+      <c r="I19" s="16" t="n"/>
+      <c r="J19" s="16" t="n"/>
+      <c r="K19" s="16" t="n"/>
+      <c r="L19" s="16" t="n"/>
+      <c r="M19" s="16" t="n"/>
+    </row>
     <row r="20" hidden="1">
       <c r="A20" t="inlineStr">
         <is>
@@ -978,6 +1172,12 @@
           <t>Cantidad</t>
         </is>
       </c>
+      <c r="H20" s="16" t="n"/>
+      <c r="I20" s="16" t="n"/>
+      <c r="J20" s="16" t="n"/>
+      <c r="K20" s="16" t="n"/>
+      <c r="L20" s="16" t="n"/>
+      <c r="M20" s="16" t="n"/>
     </row>
     <row r="21" hidden="1">
       <c r="A21" t="inlineStr">

</xml_diff>

<commit_message>
fix: embed dashboard charts as images for viewer compatibility
</commit_message>
<xml_diff>
--- a/catamarca_creditos/analisis_cartera_catamarca.xlsx
+++ b/catamarca_creditos/analisis_cartera_catamarca.xlsx
@@ -214,218 +214,56 @@
 </styleSheet>
 </file>
 
-<file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
-  <style val="10"/>
-  <chart>
-    <title>
-      <tx>
-        <rich>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-            <a:pPr>
-              <a:defRPr/>
-            </a:pPr>
-            <a:r>
-              <a:t>Estado de cartera al corte marzo 2026</a:t>
-            </a:r>
-          </a:p>
-        </rich>
-      </tx>
-    </title>
-    <plotArea>
-      <barChart>
-        <barDir val="bar"/>
-        <grouping val="clustered"/>
-        <ser>
-          <idx val="0"/>
-          <order val="0"/>
-          <tx>
-            <strRef>
-              <f>'Dashboard'!I3</f>
-            </strRef>
-          </tx>
-          <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <cat>
-            <numRef>
-              <f>'Dashboard'!$H$4:$H$7</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'Dashboard'!$I$4:$I$7</f>
-            </numRef>
-          </val>
-        </ser>
-        <gapWidth val="150"/>
-        <axId val="10"/>
-        <axId val="100"/>
-      </barChart>
-      <catAx>
-        <axId val="10"/>
-        <scaling>
-          <orientation val="minMax"/>
-        </scaling>
-        <axPos val="l"/>
-        <title>
-          <tx>
-            <rich>
-              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:pPr>
-                  <a:defRPr/>
-                </a:pPr>
-                <a:r>
-                  <a:t>Cantidad</a:t>
-                </a:r>
-              </a:p>
-            </rich>
-          </tx>
-        </title>
-        <majorTickMark val="none"/>
-        <minorTickMark val="none"/>
-        <crossAx val="100"/>
-        <lblOffset val="100"/>
-      </catAx>
-      <valAx>
-        <axId val="100"/>
-        <scaling>
-          <orientation val="minMax"/>
-        </scaling>
-        <axPos val="l"/>
-        <majorGridlines/>
-        <title>
-          <tx>
-            <rich>
-              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:pPr>
-                  <a:defRPr/>
-                </a:pPr>
-                <a:r>
-                  <a:t>Estado</a:t>
-                </a:r>
-              </a:p>
-            </rich>
-          </tx>
-        </title>
-        <majorTickMark val="none"/>
-        <minorTickMark val="none"/>
-        <crossAx val="10"/>
-      </valAx>
-    </plotArea>
-    <plotVisOnly val="1"/>
-    <dispBlanksAs val="gap"/>
-  </chart>
-</chartSpace>
-</file>
-
-<file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
-  <style val="10"/>
-  <chart>
-    <title>
-      <tx>
-        <rich>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-            <a:pPr>
-              <a:defRPr/>
-            </a:pPr>
-            <a:r>
-              <a:t>Semáforo de cartera</a:t>
-            </a:r>
-          </a:p>
-        </rich>
-      </tx>
-    </title>
-    <plotArea>
-      <pieChart>
-        <varyColors val="1"/>
-        <ser>
-          <idx val="0"/>
-          <order val="0"/>
-          <tx>
-            <strRef>
-              <f>'Dashboard'!I11</f>
-            </strRef>
-          </tx>
-          <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <cat>
-            <numRef>
-              <f>'Dashboard'!$H$12:$H$14</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'Dashboard'!$I$12:$I$14</f>
-            </numRef>
-          </val>
-        </ser>
-        <firstSliceAng val="0"/>
-      </pieChart>
-    </plotArea>
-    <legend>
-      <legendPos val="r"/>
-    </legend>
-    <plotVisOnly val="1"/>
-    <dispBlanksAs val="gap"/>
-  </chart>
-</chartSpace>
-</file>
-
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
 <wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
-      <col>10</col>
+      <col>6</col>
       <colOff>0</colOff>
       <row>1</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="4320000" cy="2520000"/>
-    <graphicFrame>
-      <nvGraphicFramePr>
-        <cNvPr id="1" name="Chart 1"/>
-        <cNvGraphicFramePr/>
-      </nvGraphicFramePr>
-      <xfrm/>
-      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
-        </a:graphicData>
-      </a:graphic>
-    </graphicFrame>
+    <ext cx="6858000" cy="3238500"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="1" name="Image 1" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId1"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
     <clientData/>
   </oneCellAnchor>
   <oneCellAnchor>
     <from>
-      <col>10</col>
+      <col>7</col>
       <colOff>0</colOff>
-      <row>17</row>
+      <row>21</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="3600000" cy="2520000"/>
-    <graphicFrame>
-      <nvGraphicFramePr>
-        <cNvPr id="2" name="Chart 2"/>
-        <cNvGraphicFramePr/>
-      </nvGraphicFramePr>
-      <xfrm/>
-      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
-        </a:graphicData>
-      </a:graphic>
-    </graphicFrame>
+    <ext cx="4381500" cy="3048000"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="2" name="Image 2" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId2"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
     <clientData/>
   </oneCellAnchor>
 </wsDr>

</xml_diff>

<commit_message>
chore: remove dashboard charts from Catamarca workbook
</commit_message>
<xml_diff>
--- a/catamarca_creditos/analisis_cartera_catamarca.xlsx
+++ b/catamarca_creditos/analisis_cartera_catamarca.xlsx
@@ -106,7 +106,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -128,6 +128,7 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="10" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -212,61 +213,6 @@
     </indexedColors>
   </colors>
 </styleSheet>
-</file>
-
-<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
-  <oneCellAnchor>
-    <from>
-      <col>6</col>
-      <colOff>0</colOff>
-      <row>1</row>
-      <rowOff>0</rowOff>
-    </from>
-    <ext cx="6858000" cy="3238500"/>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="1" name="Image 1" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId1"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
-      </spPr>
-    </pic>
-    <clientData/>
-  </oneCellAnchor>
-  <oneCellAnchor>
-    <from>
-      <col>7</col>
-      <colOff>0</colOff>
-      <row>21</row>
-      <rowOff>0</rowOff>
-    </from>
-    <ext cx="4381500" cy="3048000"/>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="2" name="Image 2" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId2"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
-      </spPr>
-    </pic>
-    <clientData/>
-  </oneCellAnchor>
-</wsDr>
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -613,7 +559,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M25"/>
+  <dimension ref="A1:O40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -621,7 +567,8 @@
     <col width="4" customWidth="1" min="3" max="3"/>
     <col width="28" customWidth="1" min="4" max="4"/>
     <col width="14" customWidth="1" min="5" max="5"/>
-    <col width="24" customWidth="1" min="8" max="8"/>
+    <col width="28" customWidth="1" min="7" max="7"/>
+    <col width="18" customWidth="1" min="8" max="8"/>
     <col width="12" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
@@ -643,16 +590,19 @@
           <t>Cruce entre Excel de depósitos y Excel de cobranzas Cecilia</t>
         </is>
       </c>
-      <c r="H2" s="15" t="inlineStr">
-        <is>
-          <t>Base gráfico estados</t>
-        </is>
-      </c>
-      <c r="I2" s="16" t="n"/>
-      <c r="J2" s="16" t="n"/>
-      <c r="K2" s="16" t="n"/>
-      <c r="L2" s="16" t="n"/>
-      <c r="M2" s="16" t="n"/>
+      <c r="G2" s="17" t="inlineStr">
+        <is>
+          <t>Resumen ejecutivo</t>
+        </is>
+      </c>
+      <c r="H2" s="17" t="n"/>
+      <c r="I2" s="17" t="n"/>
+      <c r="J2" s="17" t="n"/>
+      <c r="K2" s="17" t="n"/>
+      <c r="L2" s="17" t="n"/>
+      <c r="M2" s="17" t="n"/>
+      <c r="N2" s="17" t="n"/>
+      <c r="O2" s="17" t="n"/>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -665,20 +615,21 @@
           <t>Créditos desde 2025-12-01 y lectura de cobranza hasta marzo 2026</t>
         </is>
       </c>
-      <c r="H3" s="5" t="inlineStr">
-        <is>
-          <t>Estado</t>
-        </is>
-      </c>
-      <c r="I3" s="5" t="inlineStr">
-        <is>
-          <t>Cantidad</t>
-        </is>
-      </c>
-      <c r="J3" s="16" t="n"/>
-      <c r="K3" s="16" t="n"/>
-      <c r="L3" s="16" t="n"/>
-      <c r="M3" s="16" t="n"/>
+      <c r="G3" s="17" t="inlineStr">
+        <is>
+          <t>Créditos analizados</t>
+        </is>
+      </c>
+      <c r="H3" s="17" t="n">
+        <v>162</v>
+      </c>
+      <c r="I3" s="17" t="n"/>
+      <c r="J3" s="17" t="n"/>
+      <c r="K3" s="17" t="n"/>
+      <c r="L3" s="17" t="n"/>
+      <c r="M3" s="17" t="n"/>
+      <c r="N3" s="17" t="n"/>
+      <c r="O3" s="17" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -691,32 +642,38 @@
           <t>VERDE = al día / con cobro o finalizado | AMARILLO = sin exigibilidad clara | ROJO = mora operativa</t>
         </is>
       </c>
-      <c r="H4" s="16" t="inlineStr">
-        <is>
-          <t>Con cobro en marzo</t>
-        </is>
-      </c>
-      <c r="I4" s="16" t="n">
-        <v>59</v>
-      </c>
-      <c r="J4" s="16" t="n"/>
-      <c r="K4" s="16" t="n"/>
-      <c r="L4" s="16" t="n"/>
-      <c r="M4" s="16" t="n"/>
+      <c r="G4" s="17" t="inlineStr">
+        <is>
+          <t>Monto depositado total</t>
+        </is>
+      </c>
+      <c r="H4" s="17" t="n">
+        <v>70588070</v>
+      </c>
+      <c r="I4" s="17" t="n"/>
+      <c r="J4" s="17" t="n"/>
+      <c r="K4" s="17" t="n"/>
+      <c r="L4" s="17" t="n"/>
+      <c r="M4" s="17" t="n"/>
+      <c r="N4" s="17" t="n"/>
+      <c r="O4" s="17" t="n"/>
     </row>
     <row r="5">
-      <c r="H5" s="16" t="inlineStr">
-        <is>
-          <t>Cancelados / finalizados</t>
-        </is>
-      </c>
-      <c r="I5" s="16" t="n">
-        <v>23</v>
-      </c>
-      <c r="J5" s="16" t="n"/>
-      <c r="K5" s="16" t="n"/>
-      <c r="L5" s="16" t="n"/>
-      <c r="M5" s="16" t="n"/>
+      <c r="G5" s="17" t="inlineStr">
+        <is>
+          <t>Monto total a cobrar</t>
+        </is>
+      </c>
+      <c r="H5" s="17" t="n">
+        <v>293652000</v>
+      </c>
+      <c r="I5" s="17" t="n"/>
+      <c r="J5" s="17" t="n"/>
+      <c r="K5" s="17" t="n"/>
+      <c r="L5" s="17" t="n"/>
+      <c r="M5" s="17" t="n"/>
+      <c r="N5" s="17" t="n"/>
+      <c r="O5" s="17" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
@@ -732,18 +689,21 @@
           <t>Resumen de estado</t>
         </is>
       </c>
-      <c r="H6" s="16" t="inlineStr">
-        <is>
-          <t>Sin cobro en marzo</t>
-        </is>
-      </c>
-      <c r="I6" s="16" t="n">
-        <v>59</v>
-      </c>
-      <c r="J6" s="16" t="n"/>
-      <c r="K6" s="16" t="n"/>
-      <c r="L6" s="16" t="n"/>
-      <c r="M6" s="16" t="n"/>
+      <c r="G6" s="17" t="inlineStr">
+        <is>
+          <t>Monto cobrado en marzo</t>
+        </is>
+      </c>
+      <c r="H6" s="17" t="n">
+        <v>8740000</v>
+      </c>
+      <c r="I6" s="17" t="n"/>
+      <c r="J6" s="17" t="n"/>
+      <c r="K6" s="17" t="n"/>
+      <c r="L6" s="17" t="n"/>
+      <c r="M6" s="17" t="n"/>
+      <c r="N6" s="17" t="n"/>
+      <c r="O6" s="17" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
@@ -762,18 +722,19 @@
       <c r="E7" s="4" t="n">
         <v>78</v>
       </c>
-      <c r="H7" s="16" t="inlineStr">
-        <is>
-          <t>Sin registro en marzo</t>
-        </is>
-      </c>
-      <c r="I7" s="16" t="n">
-        <v>25</v>
-      </c>
-      <c r="J7" s="16" t="n"/>
-      <c r="K7" s="16" t="n"/>
-      <c r="L7" s="16" t="n"/>
-      <c r="M7" s="16" t="n"/>
+      <c r="G7" s="17" t="inlineStr">
+        <is>
+          <t>Mora operativa</t>
+        </is>
+      </c>
+      <c r="H7" s="17" t="n"/>
+      <c r="I7" s="17" t="n"/>
+      <c r="J7" s="17" t="n"/>
+      <c r="K7" s="17" t="n"/>
+      <c r="L7" s="17" t="n"/>
+      <c r="M7" s="17" t="n"/>
+      <c r="N7" s="17" t="n"/>
+      <c r="O7" s="17" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
@@ -792,12 +753,19 @@
       <c r="E8" s="4" t="n">
         <v>25</v>
       </c>
-      <c r="H8" s="16" t="n"/>
-      <c r="I8" s="16" t="n"/>
-      <c r="J8" s="16" t="n"/>
-      <c r="K8" s="16" t="n"/>
-      <c r="L8" s="16" t="n"/>
-      <c r="M8" s="16" t="n"/>
+      <c r="G8" s="17" t="inlineStr">
+        <is>
+          <t>% mora operativa</t>
+        </is>
+      </c>
+      <c r="H8" s="17" t="n"/>
+      <c r="I8" s="17" t="n"/>
+      <c r="J8" s="17" t="n"/>
+      <c r="K8" s="17" t="n"/>
+      <c r="L8" s="17" t="n"/>
+      <c r="M8" s="17" t="n"/>
+      <c r="N8" s="17" t="n"/>
+      <c r="O8" s="17" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
@@ -816,12 +784,15 @@
       <c r="E9" s="4" t="n">
         <v>59</v>
       </c>
-      <c r="H9" s="16" t="n"/>
-      <c r="I9" s="16" t="n"/>
-      <c r="J9" s="16" t="n"/>
-      <c r="K9" s="16" t="n"/>
-      <c r="L9" s="16" t="n"/>
-      <c r="M9" s="16" t="n"/>
+      <c r="G9" s="17" t="n"/>
+      <c r="H9" s="17" t="n"/>
+      <c r="I9" s="17" t="n"/>
+      <c r="J9" s="17" t="n"/>
+      <c r="K9" s="17" t="n"/>
+      <c r="L9" s="17" t="n"/>
+      <c r="M9" s="17" t="n"/>
+      <c r="N9" s="17" t="n"/>
+      <c r="O9" s="17" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
@@ -840,16 +811,15 @@
       <c r="E10" s="4" t="n">
         <v>23</v>
       </c>
-      <c r="H10" s="15" t="inlineStr">
-        <is>
-          <t>Base gráfico semáforo</t>
-        </is>
-      </c>
-      <c r="I10" s="16" t="n"/>
-      <c r="J10" s="16" t="n"/>
-      <c r="K10" s="16" t="n"/>
-      <c r="L10" s="16" t="n"/>
-      <c r="M10" s="16" t="n"/>
+      <c r="G10" s="17" t="n"/>
+      <c r="H10" s="17" t="n"/>
+      <c r="I10" s="17" t="n"/>
+      <c r="J10" s="17" t="n"/>
+      <c r="K10" s="17" t="n"/>
+      <c r="L10" s="17" t="n"/>
+      <c r="M10" s="17" t="n"/>
+      <c r="N10" s="17" t="n"/>
+      <c r="O10" s="17" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
@@ -868,20 +838,15 @@
       <c r="E11" s="4" t="n">
         <v>59</v>
       </c>
-      <c r="H11" s="5" t="inlineStr">
-        <is>
-          <t>Semáforo</t>
-        </is>
-      </c>
-      <c r="I11" s="5" t="inlineStr">
-        <is>
-          <t>Cantidad</t>
-        </is>
-      </c>
-      <c r="J11" s="16" t="n"/>
-      <c r="K11" s="16" t="n"/>
-      <c r="L11" s="16" t="n"/>
-      <c r="M11" s="16" t="n"/>
+      <c r="G11" s="17" t="n"/>
+      <c r="H11" s="17" t="n"/>
+      <c r="I11" s="17" t="n"/>
+      <c r="J11" s="17" t="n"/>
+      <c r="K11" s="17" t="n"/>
+      <c r="L11" s="17" t="n"/>
+      <c r="M11" s="17" t="n"/>
+      <c r="N11" s="17" t="n"/>
+      <c r="O11" s="17" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
@@ -900,18 +865,15 @@
       <c r="E12" s="4" t="n">
         <v>25</v>
       </c>
-      <c r="H12" s="16" t="inlineStr">
-        <is>
-          <t>Verde</t>
-        </is>
-      </c>
-      <c r="I12" s="16" t="n">
-        <v>78</v>
-      </c>
-      <c r="J12" s="16" t="n"/>
-      <c r="K12" s="16" t="n"/>
-      <c r="L12" s="16" t="n"/>
-      <c r="M12" s="16" t="n"/>
+      <c r="G12" s="17" t="n"/>
+      <c r="H12" s="17" t="n"/>
+      <c r="I12" s="17" t="n"/>
+      <c r="J12" s="17" t="n"/>
+      <c r="K12" s="17" t="n"/>
+      <c r="L12" s="17" t="n"/>
+      <c r="M12" s="17" t="n"/>
+      <c r="N12" s="17" t="n"/>
+      <c r="O12" s="17" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
@@ -922,75 +884,84 @@
       <c r="B13" s="10" t="n">
         <v>0.3641975308641975</v>
       </c>
-      <c r="H13" s="16" t="inlineStr">
-        <is>
-          <t>Amarillo</t>
-        </is>
-      </c>
-      <c r="I13" s="16" t="n">
-        <v>25</v>
-      </c>
-      <c r="J13" s="16" t="n"/>
-      <c r="K13" s="16" t="n"/>
-      <c r="L13" s="16" t="n"/>
-      <c r="M13" s="16" t="n"/>
+      <c r="G13" s="17" t="n"/>
+      <c r="H13" s="17" t="n"/>
+      <c r="I13" s="17" t="n"/>
+      <c r="J13" s="17" t="n"/>
+      <c r="K13" s="17" t="n"/>
+      <c r="L13" s="17" t="n"/>
+      <c r="M13" s="17" t="n"/>
+      <c r="N13" s="17" t="n"/>
+      <c r="O13" s="17" t="n"/>
     </row>
     <row r="14">
-      <c r="H14" s="16" t="inlineStr">
-        <is>
-          <t>Rojo</t>
-        </is>
-      </c>
-      <c r="I14" s="16" t="n">
-        <v>59</v>
-      </c>
-      <c r="J14" s="16" t="n"/>
-      <c r="K14" s="16" t="n"/>
-      <c r="L14" s="16" t="n"/>
-      <c r="M14" s="16" t="n"/>
+      <c r="G14" s="17" t="n"/>
+      <c r="H14" s="17" t="n"/>
+      <c r="I14" s="17" t="n"/>
+      <c r="J14" s="17" t="n"/>
+      <c r="K14" s="17" t="n"/>
+      <c r="L14" s="17" t="n"/>
+      <c r="M14" s="17" t="n"/>
+      <c r="N14" s="17" t="n"/>
+      <c r="O14" s="17" t="n"/>
     </row>
     <row r="15">
-      <c r="H15" s="16" t="n"/>
-      <c r="I15" s="16" t="n"/>
-      <c r="J15" s="16" t="n"/>
-      <c r="K15" s="16" t="n"/>
-      <c r="L15" s="16" t="n"/>
-      <c r="M15" s="16" t="n"/>
+      <c r="G15" s="17" t="n"/>
+      <c r="H15" s="17" t="n"/>
+      <c r="I15" s="17" t="n"/>
+      <c r="J15" s="17" t="n"/>
+      <c r="K15" s="17" t="n"/>
+      <c r="L15" s="17" t="n"/>
+      <c r="M15" s="17" t="n"/>
+      <c r="N15" s="17" t="n"/>
+      <c r="O15" s="17" t="n"/>
     </row>
     <row r="16">
-      <c r="H16" s="16" t="n"/>
-      <c r="I16" s="16" t="n"/>
-      <c r="J16" s="16" t="n"/>
-      <c r="K16" s="16" t="n"/>
-      <c r="L16" s="16" t="n"/>
-      <c r="M16" s="16" t="n"/>
+      <c r="G16" s="17" t="n"/>
+      <c r="H16" s="17" t="n"/>
+      <c r="I16" s="17" t="n"/>
+      <c r="J16" s="17" t="n"/>
+      <c r="K16" s="17" t="n"/>
+      <c r="L16" s="17" t="n"/>
+      <c r="M16" s="17" t="n"/>
+      <c r="N16" s="17" t="n"/>
+      <c r="O16" s="17" t="n"/>
     </row>
     <row r="17">
-      <c r="H17" s="16" t="n"/>
-      <c r="I17" s="16" t="n"/>
-      <c r="J17" s="16" t="n"/>
-      <c r="K17" s="16" t="n"/>
-      <c r="L17" s="16" t="n"/>
-      <c r="M17" s="16" t="n"/>
+      <c r="G17" s="17" t="n"/>
+      <c r="H17" s="17" t="n"/>
+      <c r="I17" s="17" t="n"/>
+      <c r="J17" s="17" t="n"/>
+      <c r="K17" s="17" t="n"/>
+      <c r="L17" s="17" t="n"/>
+      <c r="M17" s="17" t="n"/>
+      <c r="N17" s="17" t="n"/>
+      <c r="O17" s="17" t="n"/>
     </row>
     <row r="18">
-      <c r="H18" s="16" t="n"/>
-      <c r="I18" s="16" t="n"/>
-      <c r="J18" s="16" t="n"/>
-      <c r="K18" s="16" t="n"/>
-      <c r="L18" s="16" t="n"/>
-      <c r="M18" s="16" t="n"/>
+      <c r="G18" s="17" t="n"/>
+      <c r="H18" s="17" t="n"/>
+      <c r="I18" s="17" t="n"/>
+      <c r="J18" s="17" t="n"/>
+      <c r="K18" s="17" t="n"/>
+      <c r="L18" s="17" t="n"/>
+      <c r="M18" s="17" t="n"/>
+      <c r="N18" s="17" t="n"/>
+      <c r="O18" s="17" t="n"/>
     </row>
     <row r="19">
-      <c r="H19" s="16" t="n"/>
-      <c r="I19" s="16" t="n"/>
-      <c r="J19" s="16" t="n"/>
-      <c r="K19" s="16" t="n"/>
-      <c r="L19" s="16" t="n"/>
-      <c r="M19" s="16" t="n"/>
+      <c r="G19" s="17" t="n"/>
+      <c r="H19" s="17" t="n"/>
+      <c r="I19" s="17" t="n"/>
+      <c r="J19" s="17" t="n"/>
+      <c r="K19" s="17" t="n"/>
+      <c r="L19" s="17" t="n"/>
+      <c r="M19" s="17" t="n"/>
+      <c r="N19" s="17" t="n"/>
+      <c r="O19" s="17" t="n"/>
     </row>
     <row r="20" hidden="1">
-      <c r="A20" t="inlineStr">
+      <c r="A20" s="17" t="inlineStr">
         <is>
           <t>Categoría</t>
         </is>
@@ -1010,12 +981,15 @@
           <t>Cantidad</t>
         </is>
       </c>
-      <c r="H20" s="16" t="n"/>
-      <c r="I20" s="16" t="n"/>
-      <c r="J20" s="16" t="n"/>
-      <c r="K20" s="16" t="n"/>
-      <c r="L20" s="16" t="n"/>
-      <c r="M20" s="16" t="n"/>
+      <c r="G20" s="17" t="n"/>
+      <c r="H20" s="17" t="n"/>
+      <c r="I20" s="17" t="n"/>
+      <c r="J20" s="17" t="n"/>
+      <c r="K20" s="17" t="n"/>
+      <c r="L20" s="17" t="n"/>
+      <c r="M20" s="17" t="n"/>
+      <c r="N20" s="17" t="n"/>
+      <c r="O20" s="17" t="n"/>
     </row>
     <row r="21" hidden="1">
       <c r="A21" t="inlineStr">
@@ -1034,6 +1008,15 @@
       <c r="E21" t="n">
         <v>78</v>
       </c>
+      <c r="G21" s="17" t="n"/>
+      <c r="H21" s="17" t="n"/>
+      <c r="I21" s="17" t="n"/>
+      <c r="J21" s="17" t="n"/>
+      <c r="K21" s="17" t="n"/>
+      <c r="L21" s="17" t="n"/>
+      <c r="M21" s="17" t="n"/>
+      <c r="N21" s="17" t="n"/>
+      <c r="O21" s="17" t="n"/>
     </row>
     <row r="22" hidden="1">
       <c r="A22" t="inlineStr">
@@ -1052,6 +1035,15 @@
       <c r="E22" t="n">
         <v>25</v>
       </c>
+      <c r="G22" s="17" t="n"/>
+      <c r="H22" s="17" t="n"/>
+      <c r="I22" s="17" t="n"/>
+      <c r="J22" s="17" t="n"/>
+      <c r="K22" s="17" t="n"/>
+      <c r="L22" s="17" t="n"/>
+      <c r="M22" s="17" t="n"/>
+      <c r="N22" s="17" t="n"/>
+      <c r="O22" s="17" t="n"/>
     </row>
     <row r="23" hidden="1">
       <c r="A23" t="inlineStr">
@@ -1070,6 +1062,15 @@
       <c r="E23" t="n">
         <v>59</v>
       </c>
+      <c r="G23" s="17" t="n"/>
+      <c r="H23" s="17" t="n"/>
+      <c r="I23" s="17" t="n"/>
+      <c r="J23" s="17" t="n"/>
+      <c r="K23" s="17" t="n"/>
+      <c r="L23" s="17" t="n"/>
+      <c r="M23" s="17" t="n"/>
+      <c r="N23" s="17" t="n"/>
+      <c r="O23" s="17" t="n"/>
     </row>
     <row r="24" hidden="1">
       <c r="A24" t="inlineStr">
@@ -1080,6 +1081,15 @@
       <c r="B24" t="n">
         <v>25</v>
       </c>
+      <c r="G24" s="17" t="n"/>
+      <c r="H24" s="17" t="n"/>
+      <c r="I24" s="17" t="n"/>
+      <c r="J24" s="17" t="n"/>
+      <c r="K24" s="17" t="n"/>
+      <c r="L24" s="17" t="n"/>
+      <c r="M24" s="17" t="n"/>
+      <c r="N24" s="17" t="n"/>
+      <c r="O24" s="17" t="n"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -1087,13 +1097,186 @@
           <t>Mora operativa</t>
         </is>
       </c>
+      <c r="G25" s="17" t="n"/>
+      <c r="H25" s="17" t="n"/>
+      <c r="I25" s="17" t="n"/>
+      <c r="J25" s="17" t="n"/>
+      <c r="K25" s="17" t="n"/>
+      <c r="L25" s="17" t="n"/>
+      <c r="M25" s="17" t="n"/>
+      <c r="N25" s="17" t="n"/>
+      <c r="O25" s="17" t="n"/>
+    </row>
+    <row r="26">
+      <c r="G26" s="17" t="n"/>
+      <c r="H26" s="17" t="n"/>
+      <c r="I26" s="17" t="n"/>
+      <c r="J26" s="17" t="n"/>
+      <c r="K26" s="17" t="n"/>
+      <c r="L26" s="17" t="n"/>
+      <c r="M26" s="17" t="n"/>
+      <c r="N26" s="17" t="n"/>
+      <c r="O26" s="17" t="n"/>
+    </row>
+    <row r="27">
+      <c r="G27" s="17" t="n"/>
+      <c r="H27" s="17" t="n"/>
+      <c r="I27" s="17" t="n"/>
+      <c r="J27" s="17" t="n"/>
+      <c r="K27" s="17" t="n"/>
+      <c r="L27" s="17" t="n"/>
+      <c r="M27" s="17" t="n"/>
+      <c r="N27" s="17" t="n"/>
+      <c r="O27" s="17" t="n"/>
+    </row>
+    <row r="28">
+      <c r="G28" s="17" t="n"/>
+      <c r="H28" s="17" t="n"/>
+      <c r="I28" s="17" t="n"/>
+      <c r="J28" s="17" t="n"/>
+      <c r="K28" s="17" t="n"/>
+      <c r="L28" s="17" t="n"/>
+      <c r="M28" s="17" t="n"/>
+      <c r="N28" s="17" t="n"/>
+      <c r="O28" s="17" t="n"/>
+    </row>
+    <row r="29">
+      <c r="G29" s="17" t="n"/>
+      <c r="H29" s="17" t="n"/>
+      <c r="I29" s="17" t="n"/>
+      <c r="J29" s="17" t="n"/>
+      <c r="K29" s="17" t="n"/>
+      <c r="L29" s="17" t="n"/>
+      <c r="M29" s="17" t="n"/>
+      <c r="N29" s="17" t="n"/>
+      <c r="O29" s="17" t="n"/>
+    </row>
+    <row r="30">
+      <c r="G30" s="17" t="n"/>
+      <c r="H30" s="17" t="n"/>
+      <c r="I30" s="17" t="n"/>
+      <c r="J30" s="17" t="n"/>
+      <c r="K30" s="17" t="n"/>
+      <c r="L30" s="17" t="n"/>
+      <c r="M30" s="17" t="n"/>
+      <c r="N30" s="17" t="n"/>
+      <c r="O30" s="17" t="n"/>
+    </row>
+    <row r="31">
+      <c r="G31" s="17" t="n"/>
+      <c r="H31" s="17" t="n"/>
+      <c r="I31" s="17" t="n"/>
+      <c r="J31" s="17" t="n"/>
+      <c r="K31" s="17" t="n"/>
+      <c r="L31" s="17" t="n"/>
+      <c r="M31" s="17" t="n"/>
+      <c r="N31" s="17" t="n"/>
+      <c r="O31" s="17" t="n"/>
+    </row>
+    <row r="32">
+      <c r="G32" s="17" t="n"/>
+      <c r="H32" s="17" t="n"/>
+      <c r="I32" s="17" t="n"/>
+      <c r="J32" s="17" t="n"/>
+      <c r="K32" s="17" t="n"/>
+      <c r="L32" s="17" t="n"/>
+      <c r="M32" s="17" t="n"/>
+      <c r="N32" s="17" t="n"/>
+      <c r="O32" s="17" t="n"/>
+    </row>
+    <row r="33">
+      <c r="G33" s="17" t="n"/>
+      <c r="H33" s="17" t="n"/>
+      <c r="I33" s="17" t="n"/>
+      <c r="J33" s="17" t="n"/>
+      <c r="K33" s="17" t="n"/>
+      <c r="L33" s="17" t="n"/>
+      <c r="M33" s="17" t="n"/>
+      <c r="N33" s="17" t="n"/>
+      <c r="O33" s="17" t="n"/>
+    </row>
+    <row r="34">
+      <c r="G34" s="17" t="n"/>
+      <c r="H34" s="17" t="n"/>
+      <c r="I34" s="17" t="n"/>
+      <c r="J34" s="17" t="n"/>
+      <c r="K34" s="17" t="n"/>
+      <c r="L34" s="17" t="n"/>
+      <c r="M34" s="17" t="n"/>
+      <c r="N34" s="17" t="n"/>
+      <c r="O34" s="17" t="n"/>
+    </row>
+    <row r="35">
+      <c r="G35" s="17" t="n"/>
+      <c r="H35" s="17" t="n"/>
+      <c r="I35" s="17" t="n"/>
+      <c r="J35" s="17" t="n"/>
+      <c r="K35" s="17" t="n"/>
+      <c r="L35" s="17" t="n"/>
+      <c r="M35" s="17" t="n"/>
+      <c r="N35" s="17" t="n"/>
+      <c r="O35" s="17" t="n"/>
+    </row>
+    <row r="36">
+      <c r="G36" s="17" t="n"/>
+      <c r="H36" s="17" t="n"/>
+      <c r="I36" s="17" t="n"/>
+      <c r="J36" s="17" t="n"/>
+      <c r="K36" s="17" t="n"/>
+      <c r="L36" s="17" t="n"/>
+      <c r="M36" s="17" t="n"/>
+      <c r="N36" s="17" t="n"/>
+      <c r="O36" s="17" t="n"/>
+    </row>
+    <row r="37">
+      <c r="G37" s="17" t="n"/>
+      <c r="H37" s="17" t="n"/>
+      <c r="I37" s="17" t="n"/>
+      <c r="J37" s="17" t="n"/>
+      <c r="K37" s="17" t="n"/>
+      <c r="L37" s="17" t="n"/>
+      <c r="M37" s="17" t="n"/>
+      <c r="N37" s="17" t="n"/>
+      <c r="O37" s="17" t="n"/>
+    </row>
+    <row r="38">
+      <c r="G38" s="17" t="n"/>
+      <c r="H38" s="17" t="n"/>
+      <c r="I38" s="17" t="n"/>
+      <c r="J38" s="17" t="n"/>
+      <c r="K38" s="17" t="n"/>
+      <c r="L38" s="17" t="n"/>
+      <c r="M38" s="17" t="n"/>
+      <c r="N38" s="17" t="n"/>
+      <c r="O38" s="17" t="n"/>
+    </row>
+    <row r="39">
+      <c r="G39" s="17" t="n"/>
+      <c r="H39" s="17" t="n"/>
+      <c r="I39" s="17" t="n"/>
+      <c r="J39" s="17" t="n"/>
+      <c r="K39" s="17" t="n"/>
+      <c r="L39" s="17" t="n"/>
+      <c r="M39" s="17" t="n"/>
+      <c r="N39" s="17" t="n"/>
+      <c r="O39" s="17" t="n"/>
+    </row>
+    <row r="40">
+      <c r="G40" s="17" t="n"/>
+      <c r="H40" s="17" t="n"/>
+      <c r="I40" s="17" t="n"/>
+      <c r="J40" s="17" t="n"/>
+      <c r="K40" s="17" t="n"/>
+      <c r="L40" s="17" t="n"/>
+      <c r="M40" s="17" t="n"/>
+      <c r="N40" s="17" t="n"/>
+      <c r="O40" s="17" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:D1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
style: refine Catamarca dashboard presentation
</commit_message>
<xml_diff>
--- a/catamarca_creditos/analisis_cartera_catamarca.xlsx
+++ b/catamarca_creditos/analisis_cartera_catamarca.xlsx
@@ -23,7 +23,7 @@
     <numFmt numFmtId="164" formatCode="$ #,##0.00"/>
     <numFmt numFmtId="165" formatCode="yyyy-mm-dd"/>
   </numFmts>
-  <fonts count="4">
+  <fonts count="11">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -43,8 +43,49 @@
       <b val="1"/>
       <color rgb="00FFFFFF"/>
     </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="16"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="001F1F1F"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="001F1F1F"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <color rgb="001F1F1F"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="001F1F1F"/>
+      <sz val="15"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="001F1F1F"/>
+      <sz val="12"/>
+    </font>
   </fonts>
-  <fills count="7">
+  <fills count="14">
     <fill>
       <patternFill/>
     </fill>
@@ -76,6 +117,41 @@
         <fgColor rgb="00FFC7CE"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="001F3B5C"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00DCEAF7"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00EDF4FB"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFFFFF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D9EAD3"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFF2CC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F4CCCC"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -103,7 +179,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="29">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -121,6 +197,49 @@
     <xf numFmtId="165" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="8" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="9" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="10" fontId="9" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -552,247 +671,355 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E19"/>
+  <dimension ref="A1:H26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="30" customWidth="1" min="1" max="1"/>
-    <col width="22" customWidth="1" min="2" max="2"/>
-    <col width="4" customWidth="1" min="3" max="3"/>
-    <col width="28" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="3" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
     <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="3" customWidth="1" min="6" max="6"/>
+    <col width="18" customWidth="1" min="7" max="7"/>
+    <col width="16" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+    <row r="1" ht="21" customHeight="1">
+      <c r="A1" s="14" t="inlineStr">
         <is>
           <t>ANÁLISIS DE CARTERA CATAMARCA</t>
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" s="2" t="inlineStr">
+    <row r="2" ht="21" customHeight="1">
+      <c r="A2" s="15" t="inlineStr">
+        <is>
+          <t>Dashboard ejecutivo | créditos desde 2025-12-01 y cobranza hasta marzo 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="21" customHeight="1"/>
+    <row r="4" ht="21" customHeight="1">
+      <c r="A4" s="16" t="inlineStr">
         <is>
           <t>Fuente</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
+      <c r="B4" s="17" t="inlineStr">
         <is>
           <t>Cruce entre Excel de depósitos y Excel de cobranzas Cecilia</t>
         </is>
       </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="2" t="inlineStr">
-        <is>
-          <t>Corte</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>Créditos desde 2025-12-01 y lectura de cobranza hasta marzo 2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="2" t="inlineStr">
+      <c r="C4" s="4" t="n"/>
+      <c r="D4" s="4" t="n"/>
+      <c r="E4" s="4" t="n"/>
+      <c r="F4" s="4" t="n"/>
+      <c r="G4" s="4" t="n"/>
+      <c r="H4" s="4" t="n"/>
+    </row>
+    <row r="5" ht="21" customHeight="1">
+      <c r="A5" s="16" t="inlineStr">
+        <is>
+          <t>Criterio de mora</t>
+        </is>
+      </c>
+      <c r="B5" s="17" t="inlineStr">
+        <is>
+          <t>Mora operativa = crédito exigible a marzo sin cobro en marzo o sin registro en marzo, salvo cancelado/finalizado</t>
+        </is>
+      </c>
+      <c r="C5" s="4" t="n"/>
+      <c r="D5" s="4" t="n"/>
+      <c r="E5" s="4" t="n"/>
+      <c r="F5" s="4" t="n"/>
+      <c r="G5" s="4" t="n"/>
+      <c r="H5" s="4" t="n"/>
+    </row>
+    <row r="6" ht="21" customHeight="1">
+      <c r="A6" s="16" t="inlineStr">
         <is>
           <t>Semáforo</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr">
+      <c r="B6" s="17" t="inlineStr">
         <is>
           <t>VERDE = al día / con cobro o finalizado | AMARILLO = sin exigibilidad clara | ROJO = mora operativa</t>
         </is>
       </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="3" t="inlineStr">
-        <is>
-          <t>KPIs principales</t>
-        </is>
-      </c>
-      <c r="B6" s="3" t="inlineStr">
-        <is>
-          <t>Valor</t>
-        </is>
-      </c>
-      <c r="D6" s="3" t="inlineStr">
-        <is>
-          <t>Resumen de estado</t>
-        </is>
-      </c>
-      <c r="E6" s="3" t="inlineStr">
+      <c r="C6" s="4" t="n"/>
+      <c r="D6" s="4" t="n"/>
+      <c r="E6" s="4" t="n"/>
+      <c r="F6" s="4" t="n"/>
+      <c r="G6" s="4" t="n"/>
+      <c r="H6" s="4" t="n"/>
+    </row>
+    <row r="7" ht="21" customHeight="1"/>
+    <row r="8" ht="21" customHeight="1">
+      <c r="A8" s="18" t="inlineStr">
+        <is>
+          <t>Créditos analizados</t>
+        </is>
+      </c>
+      <c r="B8" s="4" t="n"/>
+      <c r="D8" s="18" t="inlineStr">
+        <is>
+          <t>Monto depositado total</t>
+        </is>
+      </c>
+      <c r="E8" s="4" t="n"/>
+      <c r="G8" s="18" t="inlineStr">
+        <is>
+          <t>Monto total a cobrar</t>
+        </is>
+      </c>
+      <c r="H8" s="4" t="n"/>
+    </row>
+    <row r="9" ht="21" customHeight="1">
+      <c r="A9" s="19" t="n">
+        <v>162</v>
+      </c>
+      <c r="B9" s="20" t="n"/>
+      <c r="D9" s="21" t="n">
+        <v>70588070</v>
+      </c>
+      <c r="E9" s="20" t="n"/>
+      <c r="G9" s="21" t="n">
+        <v>293652000</v>
+      </c>
+      <c r="H9" s="20" t="n"/>
+    </row>
+    <row r="10" ht="21" customHeight="1">
+      <c r="A10" s="20" t="n"/>
+      <c r="B10" s="20" t="n"/>
+      <c r="D10" s="20" t="n"/>
+      <c r="E10" s="20" t="n"/>
+      <c r="G10" s="20" t="n"/>
+      <c r="H10" s="20" t="n"/>
+    </row>
+    <row r="11" ht="21" customHeight="1"/>
+    <row r="12" ht="21" customHeight="1">
+      <c r="A12" s="18" t="inlineStr">
+        <is>
+          <t>Monto cobrado en marzo</t>
+        </is>
+      </c>
+      <c r="B12" s="4" t="n"/>
+      <c r="D12" s="18" t="inlineStr">
+        <is>
+          <t>Mora operativa</t>
+        </is>
+      </c>
+      <c r="E12" s="4" t="n"/>
+      <c r="G12" s="18" t="inlineStr">
+        <is>
+          <t>Monto cartera en mora</t>
+        </is>
+      </c>
+      <c r="H12" s="4" t="n"/>
+    </row>
+    <row r="13" ht="21" customHeight="1">
+      <c r="A13" s="21" t="n">
+        <v>8740000</v>
+      </c>
+      <c r="B13" s="20" t="n"/>
+      <c r="D13" s="19" t="n">
+        <v>59</v>
+      </c>
+      <c r="E13" s="20" t="n"/>
+      <c r="G13" s="21" t="n">
+        <v>106806000</v>
+      </c>
+      <c r="H13" s="20" t="n"/>
+    </row>
+    <row r="14" ht="21" customHeight="1">
+      <c r="A14" s="20" t="n"/>
+      <c r="B14" s="20" t="n"/>
+      <c r="D14" s="20" t="n"/>
+      <c r="E14" s="20" t="n"/>
+      <c r="G14" s="20" t="n"/>
+      <c r="H14" s="20" t="n"/>
+    </row>
+    <row r="15" ht="21" customHeight="1"/>
+    <row r="16" ht="21" customHeight="1">
+      <c r="A16" s="18" t="inlineStr">
+        <is>
+          <t>% con cobro en marzo</t>
+        </is>
+      </c>
+      <c r="B16" s="4" t="n"/>
+      <c r="D16" s="18" t="inlineStr">
+        <is>
+          <t>% mora operativa</t>
+        </is>
+      </c>
+      <c r="E16" s="4" t="n"/>
+      <c r="G16" s="22" t="inlineStr">
+        <is>
+          <t>Semaforización</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="21" customHeight="1">
+      <c r="A17" s="23" t="n">
+        <v>0.3641975308641975</v>
+      </c>
+      <c r="B17" s="20" t="n"/>
+      <c r="D17" s="23" t="n">
+        <v>0.3641975308641975</v>
+      </c>
+      <c r="E17" s="20" t="n"/>
+      <c r="G17" s="24" t="inlineStr">
+        <is>
+          <t>VERDE</t>
+        </is>
+      </c>
+      <c r="H17" s="25" t="n">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="18" ht="21" customHeight="1">
+      <c r="A18" s="20" t="n"/>
+      <c r="B18" s="20" t="n"/>
+      <c r="D18" s="20" t="n"/>
+      <c r="E18" s="20" t="n"/>
+      <c r="G18" s="26" t="inlineStr">
+        <is>
+          <t>AMARILLO</t>
+        </is>
+      </c>
+      <c r="H18" s="25" t="n">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="19" ht="21" customHeight="1">
+      <c r="G19" s="27" t="inlineStr">
+        <is>
+          <t>ROJO</t>
+        </is>
+      </c>
+      <c r="H19" s="25" t="n">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="20" ht="21" customHeight="1"/>
+    <row r="21" ht="21" customHeight="1"/>
+    <row r="22" ht="21" customHeight="1">
+      <c r="A22" s="22" t="inlineStr">
+        <is>
+          <t>Resumen de estado de cartera</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="21" customHeight="1">
+      <c r="A23" s="17" t="inlineStr">
+        <is>
+          <t>Cobro en marzo</t>
+        </is>
+      </c>
+      <c r="B23" s="13" t="n"/>
+      <c r="C23" s="13" t="n"/>
+      <c r="D23" s="13" t="n"/>
+      <c r="E23" s="13" t="n"/>
+      <c r="F23" s="13" t="n"/>
+      <c r="G23" s="28" t="inlineStr">
         <is>
           <t>Cantidad</t>
         </is>
       </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="4" t="inlineStr">
-        <is>
-          <t>Créditos analizados</t>
-        </is>
-      </c>
-      <c r="B7" s="4" t="n">
-        <v>162</v>
-      </c>
-      <c r="D7" s="5" t="inlineStr">
-        <is>
-          <t>VERDE</t>
-        </is>
-      </c>
-      <c r="E7" s="4" t="n">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="4" t="inlineStr">
-        <is>
-          <t>Monto depositado total</t>
-        </is>
-      </c>
-      <c r="B8" s="6" t="n">
-        <v>70588070</v>
-      </c>
-      <c r="D8" s="7" t="inlineStr">
-        <is>
-          <t>AMARILLO</t>
-        </is>
-      </c>
-      <c r="E8" s="4" t="n">
+      <c r="H23" s="25" t="n">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="24" ht="21" customHeight="1">
+      <c r="A24" s="17" t="inlineStr">
+        <is>
+          <t>Cancelados / finalizados</t>
+        </is>
+      </c>
+      <c r="B24" s="13" t="n"/>
+      <c r="C24" s="13" t="n"/>
+      <c r="D24" s="13" t="n"/>
+      <c r="E24" s="13" t="n"/>
+      <c r="F24" s="13" t="n"/>
+      <c r="G24" s="28" t="inlineStr">
+        <is>
+          <t>Cantidad</t>
+        </is>
+      </c>
+      <c r="H24" s="25" t="n">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="25" ht="21" customHeight="1">
+      <c r="A25" s="17" t="inlineStr">
+        <is>
+          <t>Sin cobro en marzo</t>
+        </is>
+      </c>
+      <c r="B25" s="13" t="n"/>
+      <c r="C25" s="13" t="n"/>
+      <c r="D25" s="13" t="n"/>
+      <c r="E25" s="13" t="n"/>
+      <c r="F25" s="13" t="n"/>
+      <c r="G25" s="28" t="inlineStr">
+        <is>
+          <t>Cantidad</t>
+        </is>
+      </c>
+      <c r="H25" s="25" t="n">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="26" ht="21" customHeight="1">
+      <c r="A26" s="17" t="inlineStr">
+        <is>
+          <t>Sin registro en marzo</t>
+        </is>
+      </c>
+      <c r="B26" s="13" t="n"/>
+      <c r="C26" s="13" t="n"/>
+      <c r="D26" s="13" t="n"/>
+      <c r="E26" s="13" t="n"/>
+      <c r="F26" s="13" t="n"/>
+      <c r="G26" s="28" t="inlineStr">
+        <is>
+          <t>Cantidad</t>
+        </is>
+      </c>
+      <c r="H26" s="25" t="n">
         <v>25</v>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" s="4" t="inlineStr">
-        <is>
-          <t>Monto total a cobrar</t>
-        </is>
-      </c>
-      <c r="B9" s="6" t="n">
-        <v>293652000</v>
-      </c>
-      <c r="D9" s="8" t="inlineStr">
-        <is>
-          <t>ROJO</t>
-        </is>
-      </c>
-      <c r="E9" s="4" t="n">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="4" t="inlineStr">
-        <is>
-          <t>Monto cobrado en marzo</t>
-        </is>
-      </c>
-      <c r="B10" s="6" t="n">
-        <v>8740000</v>
-      </c>
-      <c r="D10" s="4" t="inlineStr">
-        <is>
-          <t>Cancelados / finalizados</t>
-        </is>
-      </c>
-      <c r="E10" s="4" t="n">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="4" t="inlineStr">
-        <is>
-          <t>Clientes con cobro en marzo</t>
-        </is>
-      </c>
-      <c r="B11" s="4" t="n">
-        <v>59</v>
-      </c>
-      <c r="D11" s="4" t="inlineStr">
-        <is>
-          <t>Sin cobro en marzo</t>
-        </is>
-      </c>
-      <c r="E11" s="4" t="n">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="4" t="inlineStr">
-        <is>
-          <t>Mora operativa</t>
-        </is>
-      </c>
-      <c r="B12" s="4" t="n">
-        <v>59</v>
-      </c>
-      <c r="D12" s="4" t="inlineStr">
-        <is>
-          <t>Sin registro en marzo</t>
-        </is>
-      </c>
-      <c r="E12" s="4" t="n">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="4" t="inlineStr">
-        <is>
-          <t>Monto cartera en mora</t>
-        </is>
-      </c>
-      <c r="B13" s="6" t="n">
-        <v>106806000</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="4" t="inlineStr">
-        <is>
-          <t>% mora operativa</t>
-        </is>
-      </c>
-      <c r="B14" s="9" t="n">
-        <v>0.3641975308641975</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="D15" s="3" t="inlineStr">
-        <is>
-          <t>Resumen ejecutivo</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="D16" t="inlineStr">
-        <is>
-          <t>Créditos analizados: 162</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="D17" t="inlineStr">
-        <is>
-          <t>Clientes con cobro en marzo: 59</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="D18" t="inlineStr">
-        <is>
-          <t>Mora operativa: 59</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="D19" t="inlineStr">
-        <is>
-          <t>Cancelados / finalizados: 23</t>
-        </is>
-      </c>
-    </row>
+    <row r="27" ht="21" customHeight="1"/>
   </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="A1:E1"/>
+  <mergeCells count="27">
+    <mergeCell ref="G12:H12"/>
+    <mergeCell ref="B6:H6"/>
+    <mergeCell ref="A1:H1"/>
+    <mergeCell ref="G8:H8"/>
+    <mergeCell ref="A26:F26"/>
+    <mergeCell ref="A17:B18"/>
+    <mergeCell ref="B5:H5"/>
+    <mergeCell ref="D9:E10"/>
+    <mergeCell ref="A13:B14"/>
+    <mergeCell ref="A16:B16"/>
+    <mergeCell ref="B4:H4"/>
+    <mergeCell ref="A23:F23"/>
+    <mergeCell ref="A9:B10"/>
+    <mergeCell ref="G9:H10"/>
+    <mergeCell ref="A12:B12"/>
+    <mergeCell ref="D16:E16"/>
+    <mergeCell ref="A2:H2"/>
+    <mergeCell ref="A8:B8"/>
+    <mergeCell ref="D12:E12"/>
+    <mergeCell ref="A22:H22"/>
+    <mergeCell ref="D8:E8"/>
+    <mergeCell ref="G13:H14"/>
+    <mergeCell ref="A24:F24"/>
+    <mergeCell ref="G16:H16"/>
+    <mergeCell ref="D17:E18"/>
+    <mergeCell ref="A25:F25"/>
+    <mergeCell ref="D13:E14"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: remove redundant KPIs sheet from Catamarca workbook
</commit_message>
<xml_diff>
--- a/catamarca_creditos/analisis_cartera_catamarca.xlsx
+++ b/catamarca_creditos/analisis_cartera_catamarca.xlsx
@@ -8,9 +8,8 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="KPIs" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mora" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Consolidado" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mora" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Consolidado" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -153,7 +152,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="10">
     <border>
       <left/>
       <right/>
@@ -175,11 +174,95 @@
         <color rgb="00D9D9D9"/>
       </bottom>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00D9D9D9"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00D9D9D9"/>
+      </right>
+      <top style="thin">
+        <color rgb="00D9D9D9"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00D9D9D9"/>
+      </right>
+      <top style="thin">
+        <color rgb="00D9D9D9"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00D9D9D9"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00D9D9D9"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00D9D9D9"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="00D9D9D9"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00D9D9D9"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="00D9D9D9"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color rgb="00D9D9D9"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00D9D9D9"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color rgb="00D9D9D9"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="29">
+  <cellXfs count="34">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -241,6 +324,11 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -328,18 +416,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="T_KPIs" displayName="T_KPIs" ref="A1:B14" headerRowCount="1">
-  <autoFilter ref="A1:B14"/>
-  <tableColumns count="2">
-    <tableColumn id="1" name="KPI"/>
-    <tableColumn id="2" name="Valor"/>
-  </tableColumns>
-  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
-</table>
-</file>
-
-<file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="T_Mora" displayName="T_Mora" ref="A1:J60" headerRowCount="1">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="T_Mora" displayName="T_Mora" ref="A1:J60" headerRowCount="1">
   <autoFilter ref="A1:J60"/>
   <tableColumns count="10">
     <tableColumn id="1" name="Semáforo"/>
@@ -357,8 +434,8 @@
 </table>
 </file>
 
-<file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="T_Consolidado" displayName="T_Consolidado" ref="A1:P163" headerRowCount="1">
+<file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="T_Consolidado" displayName="T_Consolidado" ref="A1:P163" headerRowCount="1">
   <autoFilter ref="A1:P163"/>
   <tableColumns count="16">
     <tableColumn id="1" name="Semáforo"/>
@@ -710,12 +787,12 @@
           <t>Cruce entre Excel de depósitos y Excel de cobranzas Cecilia</t>
         </is>
       </c>
-      <c r="C4" s="4" t="n"/>
-      <c r="D4" s="4" t="n"/>
-      <c r="E4" s="4" t="n"/>
-      <c r="F4" s="4" t="n"/>
-      <c r="G4" s="4" t="n"/>
-      <c r="H4" s="4" t="n"/>
+      <c r="C4" s="29" t="n"/>
+      <c r="D4" s="29" t="n"/>
+      <c r="E4" s="29" t="n"/>
+      <c r="F4" s="29" t="n"/>
+      <c r="G4" s="29" t="n"/>
+      <c r="H4" s="30" t="n"/>
     </row>
     <row r="5" ht="21" customHeight="1">
       <c r="A5" s="16" t="inlineStr">
@@ -728,12 +805,12 @@
           <t>Mora operativa = crédito exigible a marzo sin cobro en marzo o sin registro en marzo, salvo cancelado/finalizado</t>
         </is>
       </c>
-      <c r="C5" s="4" t="n"/>
-      <c r="D5" s="4" t="n"/>
-      <c r="E5" s="4" t="n"/>
-      <c r="F5" s="4" t="n"/>
-      <c r="G5" s="4" t="n"/>
-      <c r="H5" s="4" t="n"/>
+      <c r="C5" s="29" t="n"/>
+      <c r="D5" s="29" t="n"/>
+      <c r="E5" s="29" t="n"/>
+      <c r="F5" s="29" t="n"/>
+      <c r="G5" s="29" t="n"/>
+      <c r="H5" s="30" t="n"/>
     </row>
     <row r="6" ht="21" customHeight="1">
       <c r="A6" s="16" t="inlineStr">
@@ -746,12 +823,12 @@
           <t>VERDE = al día / con cobro o finalizado | AMARILLO = sin exigibilidad clara | ROJO = mora operativa</t>
         </is>
       </c>
-      <c r="C6" s="4" t="n"/>
-      <c r="D6" s="4" t="n"/>
-      <c r="E6" s="4" t="n"/>
-      <c r="F6" s="4" t="n"/>
-      <c r="G6" s="4" t="n"/>
-      <c r="H6" s="4" t="n"/>
+      <c r="C6" s="29" t="n"/>
+      <c r="D6" s="29" t="n"/>
+      <c r="E6" s="29" t="n"/>
+      <c r="F6" s="29" t="n"/>
+      <c r="G6" s="29" t="n"/>
+      <c r="H6" s="30" t="n"/>
     </row>
     <row r="7" ht="21" customHeight="1"/>
     <row r="8" ht="21" customHeight="1">
@@ -760,41 +837,41 @@
           <t>Créditos analizados</t>
         </is>
       </c>
-      <c r="B8" s="4" t="n"/>
+      <c r="B8" s="30" t="n"/>
       <c r="D8" s="18" t="inlineStr">
         <is>
           <t>Monto depositado total</t>
         </is>
       </c>
-      <c r="E8" s="4" t="n"/>
+      <c r="E8" s="30" t="n"/>
       <c r="G8" s="18" t="inlineStr">
         <is>
           <t>Monto total a cobrar</t>
         </is>
       </c>
-      <c r="H8" s="4" t="n"/>
+      <c r="H8" s="30" t="n"/>
     </row>
     <row r="9" ht="21" customHeight="1">
       <c r="A9" s="19" t="n">
         <v>162</v>
       </c>
-      <c r="B9" s="20" t="n"/>
+      <c r="B9" s="31" t="n"/>
       <c r="D9" s="21" t="n">
         <v>70588070</v>
       </c>
-      <c r="E9" s="20" t="n"/>
+      <c r="E9" s="31" t="n"/>
       <c r="G9" s="21" t="n">
         <v>293652000</v>
       </c>
-      <c r="H9" s="20" t="n"/>
+      <c r="H9" s="31" t="n"/>
     </row>
     <row r="10" ht="21" customHeight="1">
-      <c r="A10" s="20" t="n"/>
-      <c r="B10" s="20" t="n"/>
-      <c r="D10" s="20" t="n"/>
-      <c r="E10" s="20" t="n"/>
-      <c r="G10" s="20" t="n"/>
-      <c r="H10" s="20" t="n"/>
+      <c r="A10" s="32" t="n"/>
+      <c r="B10" s="33" t="n"/>
+      <c r="D10" s="32" t="n"/>
+      <c r="E10" s="33" t="n"/>
+      <c r="G10" s="32" t="n"/>
+      <c r="H10" s="33" t="n"/>
     </row>
     <row r="11" ht="21" customHeight="1"/>
     <row r="12" ht="21" customHeight="1">
@@ -803,41 +880,41 @@
           <t>Monto cobrado en marzo</t>
         </is>
       </c>
-      <c r="B12" s="4" t="n"/>
+      <c r="B12" s="30" t="n"/>
       <c r="D12" s="18" t="inlineStr">
         <is>
           <t>Mora operativa</t>
         </is>
       </c>
-      <c r="E12" s="4" t="n"/>
+      <c r="E12" s="30" t="n"/>
       <c r="G12" s="18" t="inlineStr">
         <is>
           <t>Monto cartera en mora</t>
         </is>
       </c>
-      <c r="H12" s="4" t="n"/>
+      <c r="H12" s="30" t="n"/>
     </row>
     <row r="13" ht="21" customHeight="1">
       <c r="A13" s="21" t="n">
         <v>8740000</v>
       </c>
-      <c r="B13" s="20" t="n"/>
+      <c r="B13" s="31" t="n"/>
       <c r="D13" s="19" t="n">
         <v>59</v>
       </c>
-      <c r="E13" s="20" t="n"/>
+      <c r="E13" s="31" t="n"/>
       <c r="G13" s="21" t="n">
         <v>106806000</v>
       </c>
-      <c r="H13" s="20" t="n"/>
+      <c r="H13" s="31" t="n"/>
     </row>
     <row r="14" ht="21" customHeight="1">
-      <c r="A14" s="20" t="n"/>
-      <c r="B14" s="20" t="n"/>
-      <c r="D14" s="20" t="n"/>
-      <c r="E14" s="20" t="n"/>
-      <c r="G14" s="20" t="n"/>
-      <c r="H14" s="20" t="n"/>
+      <c r="A14" s="32" t="n"/>
+      <c r="B14" s="33" t="n"/>
+      <c r="D14" s="32" t="n"/>
+      <c r="E14" s="33" t="n"/>
+      <c r="G14" s="32" t="n"/>
+      <c r="H14" s="33" t="n"/>
     </row>
     <row r="15" ht="21" customHeight="1"/>
     <row r="16" ht="21" customHeight="1">
@@ -846,13 +923,13 @@
           <t>% con cobro en marzo</t>
         </is>
       </c>
-      <c r="B16" s="4" t="n"/>
+      <c r="B16" s="30" t="n"/>
       <c r="D16" s="18" t="inlineStr">
         <is>
           <t>% mora operativa</t>
         </is>
       </c>
-      <c r="E16" s="4" t="n"/>
+      <c r="E16" s="30" t="n"/>
       <c r="G16" s="22" t="inlineStr">
         <is>
           <t>Semaforización</t>
@@ -863,11 +940,11 @@
       <c r="A17" s="23" t="n">
         <v>0.3641975308641975</v>
       </c>
-      <c r="B17" s="20" t="n"/>
+      <c r="B17" s="31" t="n"/>
       <c r="D17" s="23" t="n">
         <v>0.3641975308641975</v>
       </c>
-      <c r="E17" s="20" t="n"/>
+      <c r="E17" s="31" t="n"/>
       <c r="G17" s="24" t="inlineStr">
         <is>
           <t>VERDE</t>
@@ -878,10 +955,10 @@
       </c>
     </row>
     <row r="18" ht="21" customHeight="1">
-      <c r="A18" s="20" t="n"/>
-      <c r="B18" s="20" t="n"/>
-      <c r="D18" s="20" t="n"/>
-      <c r="E18" s="20" t="n"/>
+      <c r="A18" s="32" t="n"/>
+      <c r="B18" s="33" t="n"/>
+      <c r="D18" s="32" t="n"/>
+      <c r="E18" s="33" t="n"/>
       <c r="G18" s="26" t="inlineStr">
         <is>
           <t>AMARILLO</t>
@@ -916,11 +993,11 @@
           <t>Cobro en marzo</t>
         </is>
       </c>
-      <c r="B23" s="13" t="n"/>
-      <c r="C23" s="13" t="n"/>
-      <c r="D23" s="13" t="n"/>
-      <c r="E23" s="13" t="n"/>
-      <c r="F23" s="13" t="n"/>
+      <c r="B23" s="29" t="n"/>
+      <c r="C23" s="29" t="n"/>
+      <c r="D23" s="29" t="n"/>
+      <c r="E23" s="29" t="n"/>
+      <c r="F23" s="30" t="n"/>
       <c r="G23" s="28" t="inlineStr">
         <is>
           <t>Cantidad</t>
@@ -936,11 +1013,11 @@
           <t>Cancelados / finalizados</t>
         </is>
       </c>
-      <c r="B24" s="13" t="n"/>
-      <c r="C24" s="13" t="n"/>
-      <c r="D24" s="13" t="n"/>
-      <c r="E24" s="13" t="n"/>
-      <c r="F24" s="13" t="n"/>
+      <c r="B24" s="29" t="n"/>
+      <c r="C24" s="29" t="n"/>
+      <c r="D24" s="29" t="n"/>
+      <c r="E24" s="29" t="n"/>
+      <c r="F24" s="30" t="n"/>
       <c r="G24" s="28" t="inlineStr">
         <is>
           <t>Cantidad</t>
@@ -956,11 +1033,11 @@
           <t>Sin cobro en marzo</t>
         </is>
       </c>
-      <c r="B25" s="13" t="n"/>
-      <c r="C25" s="13" t="n"/>
-      <c r="D25" s="13" t="n"/>
-      <c r="E25" s="13" t="n"/>
-      <c r="F25" s="13" t="n"/>
+      <c r="B25" s="29" t="n"/>
+      <c r="C25" s="29" t="n"/>
+      <c r="D25" s="29" t="n"/>
+      <c r="E25" s="29" t="n"/>
+      <c r="F25" s="30" t="n"/>
       <c r="G25" s="28" t="inlineStr">
         <is>
           <t>Cantidad</t>
@@ -976,11 +1053,11 @@
           <t>Sin registro en marzo</t>
         </is>
       </c>
-      <c r="B26" s="13" t="n"/>
-      <c r="C26" s="13" t="n"/>
-      <c r="D26" s="13" t="n"/>
-      <c r="E26" s="13" t="n"/>
-      <c r="F26" s="13" t="n"/>
+      <c r="B26" s="29" t="n"/>
+      <c r="C26" s="29" t="n"/>
+      <c r="D26" s="29" t="n"/>
+      <c r="E26" s="29" t="n"/>
+      <c r="F26" s="30" t="n"/>
       <c r="G26" s="28" t="inlineStr">
         <is>
           <t>Cantidad</t>
@@ -998,8 +1075,8 @@
     <mergeCell ref="A1:H1"/>
     <mergeCell ref="G8:H8"/>
     <mergeCell ref="A26:F26"/>
+    <mergeCell ref="B5:H5"/>
     <mergeCell ref="A17:B18"/>
-    <mergeCell ref="B5:H5"/>
     <mergeCell ref="D9:E10"/>
     <mergeCell ref="A13:B14"/>
     <mergeCell ref="A16:B16"/>
@@ -1031,169 +1108,6 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B14"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="45" customWidth="1" min="1" max="1"/>
-    <col width="18" customWidth="1" min="2" max="2"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="10" t="inlineStr">
-        <is>
-          <t>KPI</t>
-        </is>
-      </c>
-      <c r="B1" s="10" t="inlineStr">
-        <is>
-          <t>Valor</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="4" t="inlineStr">
-        <is>
-          <t>Créditos analizados (desde 2025-12-01)</t>
-        </is>
-      </c>
-      <c r="B2" s="4" t="n">
-        <v>162</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="4" t="inlineStr">
-        <is>
-          <t>Monto depositado total</t>
-        </is>
-      </c>
-      <c r="B3" s="6" t="n">
-        <v>70588070</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="4" t="inlineStr">
-        <is>
-          <t>Monto total a cobrar</t>
-        </is>
-      </c>
-      <c r="B4" s="6" t="n">
-        <v>293652000</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="4" t="inlineStr">
-        <is>
-          <t>Monto cobrado en marzo 2026</t>
-        </is>
-      </c>
-      <c r="B5" s="6" t="n">
-        <v>8740000</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="4" t="inlineStr">
-        <is>
-          <t>Clientes con cobro en marzo</t>
-        </is>
-      </c>
-      <c r="B6" s="4" t="n">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="4" t="inlineStr">
-        <is>
-          <t>Cancelados / finalizados</t>
-        </is>
-      </c>
-      <c r="B7" s="4" t="n">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="4" t="inlineStr">
-        <is>
-          <t>Sin cobro en marzo</t>
-        </is>
-      </c>
-      <c r="B8" s="4" t="n">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="4" t="inlineStr">
-        <is>
-          <t>Sin registro en marzo</t>
-        </is>
-      </c>
-      <c r="B9" s="4" t="n">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="4" t="inlineStr">
-        <is>
-          <t>Mora operativa</t>
-        </is>
-      </c>
-      <c r="B10" s="4" t="n">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="4" t="inlineStr">
-        <is>
-          <t>Monto total de cartera en mora operativa</t>
-        </is>
-      </c>
-      <c r="B11" s="6" t="n">
-        <v>106806000</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="4" t="inlineStr">
-        <is>
-          <t>Ticket promedio depositado</t>
-        </is>
-      </c>
-      <c r="B12" s="6" t="n">
-        <v>435728.8271604938</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="4" t="inlineStr">
-        <is>
-          <t>% con cobro en marzo</t>
-        </is>
-      </c>
-      <c r="B13" s="9" t="n">
-        <v>0.3641975308641975</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="4" t="inlineStr">
-        <is>
-          <t>% mora operativa</t>
-        </is>
-      </c>
-      <c r="B14" s="9" t="n">
-        <v>0.3641975308641975</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <tableParts count="1">
-    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
-  </tableParts>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
   <dimension ref="A1:J60"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -3747,7 +3661,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>